<commit_message>
fix(ai-sow): align feature row formatting
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-使用说明" sheetId="1" r:id="Ref95c552b72344b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-需求" sheetId="2" r:id="R38d36df26be74440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-子需求" sheetId="3" r:id="Rdce652d6205340fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-SOW主表" sheetId="4" r:id="Red87a1a08a6d4d79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-验收条件" sheetId="5" r:id="R7714d93cbbd04f44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-任务明细" sheetId="6" r:id="R221abea5730348e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06-集成点" sheetId="7" r:id="R2ae0700585df4a21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-假设清单" sheetId="8" r:id="R746d8eb9189a40c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20-项目汇总" sheetId="9" r:id="R97672f45155f4368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-系统现状" sheetId="10" r:id="R4ab59e14b277468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="91-项目参数" sheetId="11" r:id="R2bfef2b75b4e420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="92-基础人天" sheetId="12" r:id="Rc2b9c209301e487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-使用说明" sheetId="1" r:id="R79fa3a44a61c466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-需求" sheetId="2" r:id="R4b155fce7ad344c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-子需求" sheetId="3" r:id="R0e11e9e421d943d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-SOW主表" sheetId="4" r:id="R8f909793b4bd477a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-验收条件" sheetId="5" r:id="Re89c4710e0794387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-任务明细" sheetId="6" r:id="R9ba8af3ddebd4b77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06-集成点" sheetId="7" r:id="Raef57dc55099472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-假设清单" sheetId="8" r:id="R417833d062064b2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20-项目汇总" sheetId="9" r:id="Rbcb1ddf84c1248e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-系统现状" sheetId="10" r:id="Ra48c463e92a14453"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="91-项目参数" sheetId="11" r:id="R8de3c243240949b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="92-基础人天" sheetId="12" r:id="R600174cc391f414d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -322,7 +322,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="107">
+  <x:fills count="108">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -854,6 +854,11 @@
         <x:fgColor rgb="FFFFF5E3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5E3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="38">
     <x:border/>
@@ -1364,7 +1369,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="666">
+  <x:cellXfs count="675">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -3100,6 +3105,33 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="107" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -5473,8 +5505,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23908f8eb74b49d1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb630f32d9524410"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcabeb4cbf93e4926"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7d6f0ceb36f44f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5795,7 +5827,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8e6dff07d1c49b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba0859d1e85e4460"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8596,7 +8628,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf36eb22e7b54bdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76636dbf87314b72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9646,7 +9678,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b6002d81f64196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5c6f53b828b420b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9846,28 +9878,28 @@
       <x:c r="J6"/>
       <x:c r="K6"/>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="604" t="str">
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="672" t="str">
         <x:v>feature-production-scope</x:v>
       </x:c>
-      <x:c r="B7" s="604" t="str">
+      <x:c r="B7" s="672" t="str">
         <x:v>epic-platform</x:v>
       </x:c>
-      <x:c r="C7" s="604" t="str">
+      <x:c r="C7" s="672" t="str">
         <x:v>平台边界</x:v>
       </x:c>
-      <x:c r="D7" s="604" t="str">
+      <x:c r="D7" s="672" t="str">
         <x:v>生产上线范围</x:v>
       </x:c>
-      <x:c r="E7" s="604" t="str">
+      <x:c r="E7" s="672" t="str">
         <x:v>明确客户档案能力的生产上线与运营移交责任边界。</x:v>
       </x:c>
-      <x:c r="F7" s="604" t="str"/>
-      <x:c r="G7" s="604" t="str"/>
-      <x:c r="H7" s="607" t="str">
+      <x:c r="F7" s="672" t="str"/>
+      <x:c r="G7" s="672" t="str"/>
+      <x:c r="H7" s="673" t="str">
         <x:v>SOURCE_INPUT</x:v>
       </x:c>
-      <x:c r="I7" s="604" t="str"/>
+      <x:c r="I7" s="672" t="str"/>
       <x:c r="J7"/>
       <x:c r="K7"/>
     </x:row>
@@ -11147,7 +11179,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a8fb71980094c53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra58bd4ad2b9b44c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11287,11 +11319,11 @@
       </x:c>
       <x:c r="E5" s="608" t="str">
         <x:f>IF(C5="","",IFERROR(INDEX(EpicTable[需求名称],MATCH(INDEX(FeatureTable[Epic ID],MATCH(C5,FeatureTable[Feature ID],0)),EpicTable[Epic ID],0)),"来源未匹配"))</x:f>
-        <x:v>来源未匹配</x:v>
+        <x:v>客户管理</x:v>
       </x:c>
       <x:c r="F5" s="608" t="str">
         <x:f>IF(C5="","",IFERROR(INDEX(FeatureTable[子需求名称],MATCH(C5,FeatureTable[Feature ID],0)),"来源未匹配"))</x:f>
-        <x:v>来源未匹配</x:v>
+        <x:v>创建并查看客户档案</x:v>
       </x:c>
       <x:c r="G5" s="608" t="str">
         <x:f>IF(A5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[顺序]&amp;"）"&amp;AcceptanceCriterionTable[验收结果],AcceptanceCriterionTable[Story ID]=A5,"")),""))</x:f>
@@ -11336,11 +11368,11 @@
       </x:c>
       <x:c r="E6" s="608" t="str">
         <x:f>IF(C6="","",IFERROR(INDEX(EpicTable[需求名称],MATCH(INDEX(FeatureTable[Epic ID],MATCH(C6,FeatureTable[Feature ID],0)),EpicTable[Epic ID],0)),"来源未匹配"))</x:f>
-        <x:v>来源未匹配</x:v>
+        <x:v>平台边界</x:v>
       </x:c>
       <x:c r="F6" s="608" t="str">
         <x:f>IF(C6="","",IFERROR(INDEX(FeatureTable[子需求名称],MATCH(C6,FeatureTable[Feature ID],0)),"来源未匹配"))</x:f>
-        <x:v>来源未匹配</x:v>
+        <x:v>客户档案操作 API</x:v>
       </x:c>
       <x:c r="G6" s="608" t="str">
         <x:f>IF(A6="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[顺序]&amp;"）"&amp;AcceptanceCriterionTable[验收结果],AcceptanceCriterionTable[Story ID]=A6,"")),""))</x:f>
@@ -11383,11 +11415,11 @@
       </x:c>
       <x:c r="E7" s="608" t="str">
         <x:f>IF(C7="","",IFERROR(INDEX(EpicTable[需求名称],MATCH(INDEX(FeatureTable[Epic ID],MATCH(C7,FeatureTable[Feature ID],0)),EpicTable[Epic ID],0)),"来源未匹配"))</x:f>
-        <x:v>来源未匹配</x:v>
+        <x:v>平台边界</x:v>
       </x:c>
       <x:c r="F7" s="608" t="str">
         <x:f>IF(C7="","",IFERROR(INDEX(FeatureTable[子需求名称],MATCH(C7,FeatureTable[Feature ID],0)),"来源未匹配"))</x:f>
-        <x:v>来源未匹配</x:v>
+        <x:v>客户档案操作 API</x:v>
       </x:c>
       <x:c r="G7" s="608" t="str">
         <x:f>IF(A7="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[顺序]&amp;"）"&amp;AcceptanceCriterionTable[验收结果],AcceptanceCriterionTable[Story ID]=A7,"")),""))</x:f>
@@ -12688,7 +12720,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R528714014ea745c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dd8a18c0aaa46ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13403,7 +13435,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R921776aa153d4ba4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R364ccd1f1abc4a0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22241,7 +22273,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93b75909c2ea44cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dfdfeeac3374651"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23936,7 +23968,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4b3d40832e844ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ac0997c71f84b81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25226,7 +25258,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2ebe03e598e4da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ea3d7cc8a5e4f5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25597,7 +25629,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R449bd7dcba304f1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3f8a2d95b8c4b97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ai-sow): label feature coverage in as-is sheet
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -6323,7 +6323,11 @@
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
-      <c r="A44" s="618" t="inlineStr"/>
+      <c r="A44" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B44" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6358,7 +6362,11 @@
       </c>
     </row>
     <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="618" t="inlineStr"/>
+      <c r="A45" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B45" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6393,7 +6401,11 @@
       </c>
     </row>
     <row r="46" ht="45" customHeight="1">
-      <c r="A46" s="618" t="inlineStr"/>
+      <c r="A46" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B46" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6428,7 +6440,11 @@
       </c>
     </row>
     <row r="47" ht="45" customHeight="1">
-      <c r="A47" s="618" t="inlineStr"/>
+      <c r="A47" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B47" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6463,7 +6479,11 @@
       </c>
     </row>
     <row r="48" ht="45" customHeight="1">
-      <c r="A48" s="618" t="inlineStr"/>
+      <c r="A48" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B48" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6498,7 +6518,11 @@
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
-      <c r="A49" s="618" t="inlineStr"/>
+      <c r="A49" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B49" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6533,7 +6557,11 @@
       </c>
     </row>
     <row r="50" ht="45" customHeight="1">
-      <c r="A50" s="618" t="inlineStr"/>
+      <c r="A50" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B50" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6568,7 +6596,11 @@
       </c>
     </row>
     <row r="51" ht="36" customHeight="1">
-      <c r="A51" s="618" t="inlineStr"/>
+      <c r="A51" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B51" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6603,7 +6635,11 @@
       </c>
     </row>
     <row r="52" ht="36" customHeight="1">
-      <c r="A52" s="618" t="inlineStr"/>
+      <c r="A52" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B52" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6638,7 +6674,11 @@
       </c>
     </row>
     <row r="53" ht="45" customHeight="1">
-      <c r="A53" s="618" t="inlineStr"/>
+      <c r="A53" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B53" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6673,7 +6713,11 @@
       </c>
     </row>
     <row r="54" ht="45" customHeight="1">
-      <c r="A54" s="618" t="inlineStr"/>
+      <c r="A54" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B54" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>
@@ -6708,7 +6752,11 @@
       </c>
     </row>
     <row r="55" ht="36" customHeight="1">
-      <c r="A55" s="618" t="inlineStr"/>
+      <c r="A55" s="618" t="inlineStr">
+        <is>
+          <t>Feature覆盖</t>
+        </is>
+      </c>
       <c r="B55" s="618" t="inlineStr">
         <is>
           <t>COVERAGE</t>

</xml_diff>

<commit_message>
fix(ai-sow): harden e2e validation gates
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -6407,7 +6407,7 @@
       </c>
       <c r="C5" s="1053" t="inlineStr">
         <is>
-          <t>会员门户已有客户档案页面、字段校验和服务框架。</t>
+          <t>从现有客户档案页面、字段校验和服务框架开始。</t>
         </is>
       </c>
       <c r="D5" s="1057" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="C6" s="1053" t="inlineStr">
         <is>
-          <t>会员主数据保存统一会员号、基础属性和当前等级，但没有等级历史表。</t>
+          <t>复用统一会员号与基础属性表，新增等级历史和规则版本。</t>
         </is>
       </c>
       <c r="D6" s="1057" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="C7" s="1053" t="inlineStr">
         <is>
-          <t>订单服务支持线上订单基础状态流转，尚未覆盖门店订单和完整退货退款。</t>
+          <t>调整线上订单服务，扩展门店、退货退款和财务状态。</t>
         </is>
       </c>
       <c r="D7" s="1057" t="inlineStr">
@@ -6473,7 +6473,7 @@
       </c>
       <c r="C8" s="1053" t="inlineStr">
         <is>
-          <t>企业服务总线已注册 ERP 库存查询和预占接口。</t>
+          <t>接口契约保持不变，本项目完成认证、映射、适配和专项验证。</t>
         </is>
       </c>
       <c r="D8" s="1057" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="C9" s="1053" t="inlineStr">
         <is>
-          <t>企业支付网关已完成签约和生产租户开通。</t>
+          <t>支付网关平台保持不变，本项目完成配置、认证、映射和专项验证。</t>
         </is>
       </c>
       <c r="D9" s="1057" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="C10" s="1053" t="inlineStr">
         <is>
-          <t>电子发票平台已签约并提供标准开票 API。</t>
+          <t>电子发票平台保持不变，本项目完成租户设置、认证、映射和适配。</t>
         </is>
       </c>
       <c r="D10" s="1057" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="C11" s="1053" t="inlineStr">
         <is>
-          <t>现有 Kubernetes 集群、制品库和 CI/CD 流水线承载会员门户与订单服务。</t>
+          <t>在现有集群与流水线中增加应用配置、发布步骤、切换和回滚清单。</t>
         </is>
       </c>
       <c r="D11" s="1057" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="C12" s="1053" t="inlineStr">
         <is>
-          <t>现有身份平台提供员工与门店角色控制，授权中心保存会员授权记录。</t>
+          <t>现有授权、撤回、查询与审计能力已完整覆盖本期目标。</t>
         </is>
       </c>
       <c r="D12" s="1057" t="inlineStr">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C13" s="1053" t="inlineStr">
         <is>
-          <t>消息中心已消费标准订单事件并通过短信、App Push 发送通知。</t>
+          <t>标准订单事件和现有通知通道已完整覆盖本期通知目标。</t>
         </is>
       </c>
       <c r="D13" s="1057" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="C14" s="1053" t="inlineStr">
         <is>
-          <t>平台已采集应用日志、指标与链路，但缺少新订单指标和财务批处理告警。</t>
+          <t>复用日志、指标和链路平台，新增订单与财务作业监控。</t>
         </is>
       </c>
       <c r="D14" s="1057" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="C15" s="1053" t="inlineStr">
         <is>
-          <t>一期已有 API 自动化框架、订单基础用例和兼容矩阵。</t>
+          <t>调整既有测试框架、测试用例、测试脚本、兼容矩阵与负载模型。</t>
         </is>
       </c>
       <c r="D15" s="1057" t="inlineStr">

</xml_diff>

<commit_message>
fix(ai-sow): support legacy Excel SOW formulas
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -5003,10 +5003,10 @@
     <tableColumn id="3" name="故事名称"/>
     <tableColumn id="4" name="UAT适用"/>
     <tableColumn id="5" name="验收条件">
-      <calculatedColumnFormula>IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C5,"")),""))</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C5,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" name="任务明细">
-      <calculatedColumnFormula>IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C5,"")),""))</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C5,"• "&amp;TaskTable[任务名称],"")),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" name="人天">
       <calculatedColumnFormula>IF(C5="","",CEILING(SUMIF(TaskTable[故事名称],C5,TaskTable[人天小计]),INDEX(ProjectParameterTable[值],MATCH("ROUND_STORY",ProjectParameterTable[参数代码],0))))</calculatedColumnFormula>
@@ -11711,11 +11711,11 @@
         </is>
       </c>
       <c r="E5" s="926">
-        <f>IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C5,"")),""))</f>
+        <f t="array" ref="E5">IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C5,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F5" s="928">
-        <f>IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C5,"")),""))</f>
+        <f t="array" ref="F5">IF(C5="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C5,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G5" s="929">
@@ -11749,11 +11749,11 @@
         </is>
       </c>
       <c r="E6" s="926">
-        <f>IF(C6="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C6,"")),""))</f>
+        <f t="array" ref="E6">IF(C6="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C6,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F6" s="928">
-        <f>IF(C6="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C6,"")),""))</f>
+        <f t="array" ref="F6">IF(C6="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C6,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G6" s="929">
@@ -11787,11 +11787,11 @@
         </is>
       </c>
       <c r="E7" s="926">
-        <f>IF(C7="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C7,"")),""))</f>
+        <f t="array" ref="E7">IF(C7="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C7,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F7" s="928">
-        <f>IF(C7="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C7,"")),""))</f>
+        <f t="array" ref="F7">IF(C7="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C7,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G7" s="929">
@@ -11829,11 +11829,11 @@
         </is>
       </c>
       <c r="E8" s="926">
-        <f>IF(C8="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C8,"")),""))</f>
+        <f t="array" ref="E8">IF(C8="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C8,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F8" s="928">
-        <f>IF(C8="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C8,"")),""))</f>
+        <f t="array" ref="F8">IF(C8="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C8,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G8" s="929">
@@ -11871,11 +11871,11 @@
         </is>
       </c>
       <c r="E9" s="926">
-        <f>IF(C9="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C9,"")),""))</f>
+        <f t="array" ref="E9">IF(C9="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C9,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F9" s="928">
-        <f>IF(C9="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C9,"")),""))</f>
+        <f t="array" ref="F9">IF(C9="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C9,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G9" s="929">
@@ -11909,11 +11909,11 @@
         </is>
       </c>
       <c r="E10" s="926">
-        <f>IF(C10="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C10,"")),""))</f>
+        <f t="array" ref="E10">IF(C10="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C10,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F10" s="928">
-        <f>IF(C10="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C10,"")),""))</f>
+        <f t="array" ref="F10">IF(C10="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C10,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G10" s="929">
@@ -11947,11 +11947,11 @@
         </is>
       </c>
       <c r="E11" s="926">
-        <f>IF(C11="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C11,"")),""))</f>
+        <f t="array" ref="E11">IF(C11="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C11,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F11" s="928">
-        <f>IF(C11="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C11,"")),""))</f>
+        <f t="array" ref="F11">IF(C11="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C11,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G11" s="929">
@@ -11989,11 +11989,11 @@
         </is>
       </c>
       <c r="E12" s="926">
-        <f>IF(C12="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C12,"")),""))</f>
+        <f t="array" ref="E12">IF(C12="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C12,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F12" s="928">
-        <f>IF(C12="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C12,"")),""))</f>
+        <f t="array" ref="F12">IF(C12="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C12,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G12" s="929">
@@ -12027,11 +12027,11 @@
         </is>
       </c>
       <c r="E13" s="926">
-        <f>IF(C13="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C13,"")),""))</f>
+        <f t="array" ref="E13">IF(C13="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C13,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F13" s="928">
-        <f>IF(C13="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C13,"")),""))</f>
+        <f t="array" ref="F13">IF(C13="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C13,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G13" s="929">
@@ -12069,11 +12069,11 @@
         </is>
       </c>
       <c r="E14" s="926">
-        <f>IF(C14="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C14,"")),""))</f>
+        <f t="array" ref="E14">IF(C14="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C14,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F14" s="928">
-        <f>IF(C14="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C14,"")),""))</f>
+        <f t="array" ref="F14">IF(C14="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C14,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G14" s="929">
@@ -12107,11 +12107,11 @@
         </is>
       </c>
       <c r="E15" s="926">
-        <f>IF(C15="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C15,"")),""))</f>
+        <f t="array" ref="E15">IF(C15="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C15,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F15" s="928">
-        <f>IF(C15="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C15,"")),""))</f>
+        <f t="array" ref="F15">IF(C15="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C15,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G15" s="929">
@@ -12145,11 +12145,11 @@
         </is>
       </c>
       <c r="E16" s="926">
-        <f>IF(C16="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C16,"")),""))</f>
+        <f t="array" ref="E16">IF(C16="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C16,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F16" s="928">
-        <f>IF(C16="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C16,"")),""))</f>
+        <f t="array" ref="F16">IF(C16="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C16,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G16" s="929">
@@ -12183,11 +12183,11 @@
         </is>
       </c>
       <c r="E17" s="926">
-        <f>IF(C17="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C17,"")),""))</f>
+        <f t="array" ref="E17">IF(C17="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C17,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F17" s="928">
-        <f>IF(C17="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C17,"")),""))</f>
+        <f t="array" ref="F17">IF(C17="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C17,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G17" s="929">
@@ -12225,11 +12225,11 @@
         </is>
       </c>
       <c r="E18" s="926">
-        <f>IF(C18="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C18,"")),""))</f>
+        <f t="array" ref="E18">IF(C18="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C18,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F18" s="928">
-        <f>IF(C18="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C18,"")),""))</f>
+        <f t="array" ref="F18">IF(C18="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C18,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G18" s="929">
@@ -12263,11 +12263,11 @@
         </is>
       </c>
       <c r="E19" s="926">
-        <f>IF(C19="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C19,"")),""))</f>
+        <f t="array" ref="E19">IF(C19="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C19,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F19" s="928">
-        <f>IF(C19="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C19,"")),""))</f>
+        <f t="array" ref="F19">IF(C19="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C19,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G19" s="929">
@@ -12301,11 +12301,11 @@
         </is>
       </c>
       <c r="E20" s="926">
-        <f>IF(C20="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C20,"")),""))</f>
+        <f t="array" ref="E20">IF(C20="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C20,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F20" s="928">
-        <f>IF(C20="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C20,"")),""))</f>
+        <f t="array" ref="F20">IF(C20="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C20,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G20" s="929">
@@ -12343,11 +12343,11 @@
         </is>
       </c>
       <c r="E21" s="926">
-        <f>IF(C21="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C21,"")),""))</f>
+        <f t="array" ref="E21">IF(C21="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C21,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F21" s="928">
-        <f>IF(C21="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C21,"")),""))</f>
+        <f t="array" ref="F21">IF(C21="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C21,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G21" s="929">
@@ -12385,11 +12385,11 @@
         </is>
       </c>
       <c r="E22" s="926">
-        <f>IF(C22="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C22,"")),""))</f>
+        <f t="array" ref="E22">IF(C22="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C22,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F22" s="928">
-        <f>IF(C22="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C22,"")),""))</f>
+        <f t="array" ref="F22">IF(C22="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C22,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G22" s="929">
@@ -12427,11 +12427,11 @@
         </is>
       </c>
       <c r="E23" s="926">
-        <f>IF(C23="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C23,"")),""))</f>
+        <f t="array" ref="E23">IF(C23="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C23,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F23" s="928">
-        <f>IF(C23="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C23,"")),""))</f>
+        <f t="array" ref="F23">IF(C23="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C23,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G23" s="929">
@@ -12469,11 +12469,11 @@
         </is>
       </c>
       <c r="E24" s="926">
-        <f>IF(C24="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C24,"")),""))</f>
+        <f t="array" ref="E24">IF(C24="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C24,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F24" s="928">
-        <f>IF(C24="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C24,"")),""))</f>
+        <f t="array" ref="F24">IF(C24="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C24,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G24" s="929">
@@ -12507,11 +12507,11 @@
         </is>
       </c>
       <c r="E25" s="926">
-        <f>IF(C25="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C25,"")),""))</f>
+        <f t="array" ref="E25">IF(C25="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C25,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F25" s="928">
-        <f>IF(C25="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C25,"")),""))</f>
+        <f t="array" ref="F25">IF(C25="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C25,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G25" s="929">
@@ -12545,11 +12545,11 @@
         </is>
       </c>
       <c r="E26" s="926">
-        <f>IF(C26="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C26,"")),""))</f>
+        <f t="array" ref="E26">IF(C26="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C26,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F26" s="928">
-        <f>IF(C26="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C26,"")),""))</f>
+        <f t="array" ref="F26">IF(C26="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C26,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G26" s="929">
@@ -12583,11 +12583,11 @@
         </is>
       </c>
       <c r="E27" s="926">
-        <f>IF(C27="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER(AcceptanceCriterionTable[验收条件名称],AcceptanceCriterionTable[故事名称]=C27,"")),""))</f>
+        <f t="array" ref="E27">IF(C27="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(AcceptanceCriterionTable[故事名称]=C27,"• "&amp;AcceptanceCriterionTable[验收条件名称],"")),""))</f>
         <v/>
       </c>
       <c r="F27" s="928">
-        <f>IF(C27="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,_xlfn._xlws.FILTER("• "&amp;TaskTable[任务名称],TaskTable[故事名称]=C27,"")),""))</f>
+        <f t="array" ref="F27">IF(C27="","",IFERROR(_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(TaskTable[故事名称]=C27,"• "&amp;TaskTable[任务名称],"")),""))</f>
         <v/>
       </c>
       <c r="G27" s="929">
@@ -13679,7 +13679,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -14463,7 +14463,7 @@
     <row r="103" s="1025"/>
     <row r="104" s="1025"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -18163,7 +18163,7 @@
     <row r="503" s="1025"/>
     <row r="504" s="1025"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
@@ -18710,7 +18710,7 @@
     <row r="103" s="1025"/>
     <row r="104" s="1025"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -20557,7 +20557,7 @@
       <c r="F100" s="948" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
fix(ai-sow): allow protected sheet filters and sorting
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -13679,7 +13679,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -14463,7 +14463,7 @@
     <row r="103" s="1025"/>
     <row r="104" s="1025"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -18163,7 +18163,7 @@
     <row r="503" s="1025"/>
     <row r="504" s="1025"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
@@ -18710,7 +18710,7 @@
     <row r="103" s="1025"/>
     <row r="104" s="1025"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -20557,7 +20557,7 @@
       <c r="F100" s="948" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
feat(ai-sow): accelerate reviews and simplify delivery
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -6202,7 +6202,7 @@
       </c>
       <c r="B45" s="1040" t="inlineStr">
         <is>
-          <t>e82bed56bfdeef7657145d894f813eec584179277812152eaa0b93cf36cf26ce</t>
+          <t>f53080d649a2f8d30feb355c7054ee39b5db643556d769be9fa9019700aae0ee</t>
         </is>
       </c>
       <c r="C45" s="1041" t="n"/>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="B48" s="1040" t="inlineStr">
         <is>
-          <t>0aeb3baff7024ba001b3206c687c3f35bb09436c579f4be4de14cd178d3271ed</t>
+          <t>aac75df69d3dbcc48e4a15a9cf3dee699c95246b9ff062e662d93aaf69218228</t>
         </is>
       </c>
       <c r="C48" s="1041" t="n"/>

</xml_diff>

<commit_message>
fix(ai-sow): expand wrapped workbook rows
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
+++ b/plugins/ai-sow/docs/reference/SOW估算与生成示例_v1.3.xlsx
@@ -10482,7 +10482,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="1025">
+    <row r="5" ht="49" customHeight="1" s="1025">
       <c r="A5" s="1058" t="inlineStr">
         <is>
           <t>会员与客户管理</t>
@@ -10514,7 +10514,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="1025">
+    <row r="6" ht="49" customHeight="1" s="1025">
       <c r="A6" s="1058" t="inlineStr">
         <is>
           <t>订单与履约</t>
@@ -10546,7 +10546,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="1025">
+    <row r="7" ht="49" customHeight="1" s="1025">
       <c r="A7" s="1058" t="inlineStr">
         <is>
           <t>全渠道运营</t>
@@ -10578,7 +10578,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="1025">
+    <row r="8" ht="34" customHeight="1" s="1025">
       <c r="A8" s="1058" t="inlineStr">
         <is>
           <t>财务结算与经营分析</t>
@@ -10610,7 +10610,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="1025">
+    <row r="9" ht="34" customHeight="1" s="1025">
       <c r="A9" s="1058" t="inlineStr">
         <is>
           <t>平台与服务边界</t>
@@ -10642,7 +10642,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" s="1025">
+    <row r="10" ht="34" customHeight="1" s="1025">
       <c r="A10" s="1058" t="inlineStr">
         <is>
           <t>上线与质量保障</t>
@@ -10912,7 +10912,7 @@
       </c>
       <c r="G5" s="1058" t="inlineStr"/>
     </row>
-    <row r="6" ht="34" customHeight="1" s="1025">
+    <row r="6" ht="49" customHeight="1" s="1025">
       <c r="A6" s="1058" t="inlineStr">
         <is>
           <t>会员与客户管理</t>
@@ -11176,7 +11176,7 @@
       </c>
       <c r="G13" s="1058" t="inlineStr"/>
     </row>
-    <row r="14" ht="34" customHeight="1" s="1025">
+    <row r="14" ht="49" customHeight="1" s="1025">
       <c r="A14" s="1058" t="inlineStr">
         <is>
           <t>财务结算与经营分析</t>
@@ -11275,7 +11275,7 @@
       </c>
       <c r="G16" s="1058" t="inlineStr"/>
     </row>
-    <row r="17" ht="34" customHeight="1" s="1025">
+    <row r="17" ht="94" customHeight="1" s="1025">
       <c r="A17" s="1058" t="inlineStr">
         <is>
           <t>平台与服务边界</t>
@@ -11728,7 +11728,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1" s="1025">
+    <row r="6" ht="49" customHeight="1" s="1025">
       <c r="A6" s="926">
         <f>IF(B6="","",IFERROR(INDEX(FeatureTable[需求名称],MATCH(B6,FeatureTable[子需求名称],0)),"来源未匹配"))</f>
         <v/>
@@ -12162,7 +12162,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1" s="1025">
+    <row r="17" ht="49" customHeight="1" s="1025">
       <c r="A17" s="926">
         <f>IF(B17="","",IFERROR(INDEX(FeatureTable[需求名称],MATCH(B17,FeatureTable[子需求名称],0)),"来源未匹配"))</f>
         <v/>
@@ -12242,7 +12242,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1" s="1025">
+    <row r="19" ht="49" customHeight="1" s="1025">
       <c r="A19" s="926">
         <f>IF(B19="","",IFERROR(INDEX(FeatureTable[需求名称],MATCH(B19,FeatureTable[子需求名称],0)),"来源未匹配"))</f>
         <v/>
@@ -12322,7 +12322,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1" s="1025">
+    <row r="21" ht="49" customHeight="1" s="1025">
       <c r="A21" s="926">
         <f>IF(B21="","",IFERROR(INDEX(FeatureTable[需求名称],MATCH(B21,FeatureTable[子需求名称],0)),"来源未匹配"))</f>
         <v/>
@@ -12364,7 +12364,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1" s="1025">
+    <row r="22" ht="49" customHeight="1" s="1025">
       <c r="A22" s="926">
         <f>IF(B22="","",IFERROR(INDEX(FeatureTable[需求名称],MATCH(B22,FeatureTable[子需求名称],0)),"来源未匹配"))</f>
         <v/>
@@ -14646,7 +14646,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1" s="1025">
+    <row r="5" ht="49" customHeight="1" s="1025">
       <c r="A5" s="944">
         <f>IF(C5="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C5,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -14717,7 +14717,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1" s="1025">
+    <row r="6" ht="49" customHeight="1" s="1025">
       <c r="A6" s="944">
         <f>IF(C6="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C6,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -14784,7 +14784,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1" s="1025">
+    <row r="7" ht="49" customHeight="1" s="1025">
       <c r="A7" s="944">
         <f>IF(C7="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C7,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15052,7 +15052,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1" s="1025">
+    <row r="11" ht="49" customHeight="1" s="1025">
       <c r="A11" s="944">
         <f>IF(C11="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C11,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15186,7 +15186,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1" s="1025">
+    <row r="13" ht="49" customHeight="1" s="1025">
       <c r="A13" s="944">
         <f>IF(C13="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C13,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15320,7 +15320,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1" s="1025">
+    <row r="15" ht="49" customHeight="1" s="1025">
       <c r="A15" s="944">
         <f>IF(C15="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C15,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15387,7 +15387,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1" s="1025">
+    <row r="16" ht="49" customHeight="1" s="1025">
       <c r="A16" s="944">
         <f>IF(C16="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C16,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15454,7 +15454,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="38" customHeight="1" s="1025">
+    <row r="17" ht="49" customHeight="1" s="1025">
       <c r="A17" s="944">
         <f>IF(C17="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C17,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15651,7 +15651,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="38" customHeight="1" s="1025">
+    <row r="20" ht="49" customHeight="1" s="1025">
       <c r="A20" s="944">
         <f>IF(C20="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C20,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -15848,7 +15848,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="38" customHeight="1" s="1025">
+    <row r="23" ht="49" customHeight="1" s="1025">
       <c r="A23" s="944">
         <f>IF(C23="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C23,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16171,7 +16171,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="38" customHeight="1" s="1025">
+    <row r="28" ht="49" customHeight="1" s="1025">
       <c r="A28" s="944">
         <f>IF(C28="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C28,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16301,7 +16301,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="38" customHeight="1" s="1025">
+    <row r="30" ht="49" customHeight="1" s="1025">
       <c r="A30" s="944">
         <f>IF(C30="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C30,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16431,7 +16431,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="38" customHeight="1" s="1025">
+    <row r="32" ht="49" customHeight="1" s="1025">
       <c r="A32" s="944">
         <f>IF(C32="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C32,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16498,7 +16498,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="38" customHeight="1" s="1025">
+    <row r="33" ht="49" customHeight="1" s="1025">
       <c r="A33" s="944">
         <f>IF(C33="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C33,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16565,7 +16565,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="38" customHeight="1" s="1025">
+    <row r="34" ht="49" customHeight="1" s="1025">
       <c r="A34" s="944">
         <f>IF(C34="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C34,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16636,7 +16636,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="38" customHeight="1" s="1025">
+    <row r="35" ht="49" customHeight="1" s="1025">
       <c r="A35" s="944">
         <f>IF(C35="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C35,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16707,7 +16707,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="38" customHeight="1" s="1025">
+    <row r="36" ht="49" customHeight="1" s="1025">
       <c r="A36" s="944">
         <f>IF(C36="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C36,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16774,7 +16774,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="38" customHeight="1" s="1025">
+    <row r="37" ht="49" customHeight="1" s="1025">
       <c r="A37" s="944">
         <f>IF(C37="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C37,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -16967,7 +16967,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="38" customHeight="1" s="1025">
+    <row r="40" ht="49" customHeight="1" s="1025">
       <c r="A40" s="944">
         <f>IF(C40="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C40,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -17038,7 +17038,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="38" customHeight="1" s="1025">
+    <row r="41" ht="49" customHeight="1" s="1025">
       <c r="A41" s="944">
         <f>IF(C41="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C41,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -17168,7 +17168,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="38" customHeight="1" s="1025">
+    <row r="43" ht="49" customHeight="1" s="1025">
       <c r="A43" s="944">
         <f>IF(C43="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C43,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -17298,7 +17298,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="38" customHeight="1" s="1025">
+    <row r="45" ht="49" customHeight="1" s="1025">
       <c r="A45" s="944">
         <f>IF(C45="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C45,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -17495,7 +17495,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="38" customHeight="1" s="1025">
+    <row r="48" ht="49" customHeight="1" s="1025">
       <c r="A48" s="944">
         <f>IF(C48="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C48,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -17566,7 +17566,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="38" customHeight="1" s="1025">
+    <row r="49" ht="49" customHeight="1" s="1025">
       <c r="A49" s="944">
         <f>IF(C49="","",IFERROR(INDEX(SOWStoryTable[需求名称],MATCH(C49,SOWStoryTable[故事名称],0)),"来源未匹配"))</f>
         <v/>
@@ -18920,7 +18920,7 @@
       <c r="H7" s="1049" t="n"/>
       <c r="I7" s="1049" t="n"/>
     </row>
-    <row r="8" ht="38" customHeight="1" s="1025">
+    <row r="8" ht="49" customHeight="1" s="1025">
       <c r="A8" s="1060" t="inlineStr">
         <is>
           <t>支付网关退款认证可能延迟</t>

</xml_diff>